<commit_message>
Revise Fullscript header navigation mockup
</commit_message>
<xml_diff>
--- a/outputs/01a062b4-9ceb-7123-8739-1154f7acbf63/Rebekahs-Phase-Two-Ecommerce-Workbook.xlsx
+++ b/outputs/01a062b4-9ceb-7123-8739-1154f7acbf63/Rebekahs-Phase-Two-Ecommerce-Workbook.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Set" sheetId="1" r:id="R3bc72fa3ccb04650"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates &amp; Global" sheetId="2" r:id="R67ef9a37e9d649c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product &amp; Content" sheetId="3" r:id="R76c82fb7296b4c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions &amp; Access" sheetId="4" r:id="Rd24ced66dc874232"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="5" r:id="Rbeefdf63a1024a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA &amp; Launch Gates" sheetId="6" r:id="Rdcabf31f17b34268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope &amp; Costs" sheetId="7" r:id="R4213cf14b2f24db6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version Register" sheetId="8" r:id="Rebbaeb6c8cab4d08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training &amp; Handoff" sheetId="9" r:id="Rc8fa24ea7db54d34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pre-Staging Packet" sheetId="10" r:id="R306416158d874513"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Set" sheetId="1" r:id="R5c6d75c39a794386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates &amp; Global" sheetId="2" r:id="R3a4529c91f1944b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product &amp; Content" sheetId="3" r:id="R35bf7142d8934b43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions &amp; Access" sheetId="4" r:id="R8fc8e98234684a53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="5" r:id="Re92f0150b0c84bc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA &amp; Launch Gates" sheetId="6" r:id="Rb644898d6f904b8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope &amp; Costs" sheetId="7" r:id="Rd940e3ba00864c2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version Register" sheetId="8" r:id="Rfdc6f91174ce4ef8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training &amp; Handoff" sheetId="9" r:id="R6dc212dfa5d24ff8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pre-Staging Packet" sheetId="10" r:id="R8b7a442aa9e84ddc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1399,10 +1399,10 @@
         <x:v>Internally approved</x:v>
       </x:c>
       <x:c r="D3" s="13" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Awaiting client</x:v>
+        <x:v>Awaiting internal</x:v>
       </x:c>
       <x:c r="F3" s="13" t="n">
         <x:v>1</x:v>
@@ -1417,7 +1417,7 @@
         <x:v>Current gate</x:v>
       </x:c>
       <x:c r="J3" s="13" t="str">
-        <x:v>Rebekah confirms exact Shop/Catalog v1.9</x:v>
+        <x:v>Todd reviews Header + Footer v1.6</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
@@ -1466,7 +1466,7 @@
         <x:v>Sitewide</x:v>
       </x:c>
       <x:c r="E6" s="131" t="str">
-        <x:v>Client Approved</x:v>
+        <x:v>Revision Needed</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:v>Local mockup</x:v>
@@ -1481,7 +1481,7 @@
         <x:v>Store entry, internal links, policy links, responsive navigation, account/cart indexation.</x:v>
       </x:c>
       <x:c r="J6" s="20" t="str">
-        <x:v>Exact Header + Footer Ecommerce Add-On v1.5 was approved by Todd and approved by Rebekah on September 2, 2026. Production Online Store links will use /shop/. Any later design change requires v1.6 and new exact-version approval.</x:v>
+        <x:v>v1.6 moves Shop Fullscript out of the In-Store Products submenu and places it directly on the main navigation bar. Awaiting Todd review; Rebekah's prior v1.5 approval does not transfer to this revision.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="80" customHeight="1">
@@ -1701,7 +1701,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaa003b77c1443f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R219c49033ba74406"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2426,7 +2426,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22babf813ce44133"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1636eeb024844052"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3023,7 +3023,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6078fd4ee54b4d6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb596118607a44ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3654,7 +3654,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf73adf8268024b41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R464a6fcb44174cbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3973,7 +3973,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R709b8746eb9a4720"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e6ecb76ab6d4b8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4661,7 +4661,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0b61bc3ab3c483a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra229b5909eb64d1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5117,7 +5117,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9af311c769347af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R464e7707eadd4789"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5231,25 +5231,25 @@
         <x:v>Header + Footer Ecommerce Add-On</x:v>
       </x:c>
       <x:c r="C6" s="57" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="D6" s="55" t="str">
-        <x:v>online-store-header-footer-add-on-v1.5.html</x:v>
+        <x:v>online-store-header-footer-add-on-v1.6.html</x:v>
       </x:c>
       <x:c r="E6" s="134" t="str">
-        <x:v>Client Approved</x:v>
+        <x:v>Revision Needed</x:v>
       </x:c>
       <x:c r="F6" s="55" t="str">
-        <x:v>Approved by Todd</x:v>
+        <x:v>Awaiting Todd</x:v>
       </x:c>
       <x:c r="G6" s="134" t="str">
-        <x:v>Approved by Rebekah 2026-09-02</x:v>
+        <x:v>Pending Rebekah</x:v>
       </x:c>
       <x:c r="H6" s="57" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.7</x:v>
       </x:c>
       <x:c r="I6" s="55" t="str">
-        <x:v>Exact v1.5 approved by Todd and Rebekah on September 2, 2026. Production Online Store links will use /shop/. Any later design change requires v1.6 and new exact-version approval.</x:v>
+        <x:v>Shop Fullscript is now a direct main-menu item rather than a child of In-Store Products. The approved responsive header, ecommerce utility row, and footer are preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
@@ -5956,7 +5956,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8af852c72f24d80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re100dbf20d7f4532"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>